<commit_message>
feat: update Supabase dependencies and add migration script for product images
- Added @supabase/supabase-js dependency to package.json and package-lock.json.
- Created a new script (migrate-images.js) to migrate existing local product images to Supabase Storage and update their URLs in the database.
- Updated Excel templates in the frontend.
- Removed 'qty' translation from LanguageContext.
- Added unit price to sales transaction in SalesPage.
</commit_message>
<xml_diff>
--- a/frontend/public/Excels Templates/TransferTemplates.xlsx
+++ b/frontend/public/Excels Templates/TransferTemplates.xlsx
@@ -1,64 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MyWork\Yogini Arts\Website\YoginiArts\frontend\public\Excels Templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7FB524E-FC5B-4760-ACBE-A5A9E9A592DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{43EF93C9-C5B1-41B9-BCC7-E1113705257E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13920" xr2:uid="{56CB4373-1968-40B0-B961-900DE774D5A0}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="20 Package" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>Sent to Yukesh 60 RMB</t>
-  </si>
-  <si>
     <t>Image</t>
   </si>
   <si>
-    <t>Product name</t>
+    <t>Product Name</t>
   </si>
   <si>
-    <t>Bar code</t>
+    <t>Bar Code</t>
   </si>
   <si>
-    <t>Weight</t>
+    <t>Transferred To</t>
   </si>
   <si>
-    <t>Size</t>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Sent to Yukesh 60 RMB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,11 +49,9 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="13"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -81,19 +60,8 @@
       <name val="Calibri(BODY)"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri(body)"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <color theme="0"/>
-      <name val="Calibri(BODY)"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -102,24 +70,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF162830"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF720E20"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -129,52 +84,56 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyProtection="0">
-      <alignment horizontal="center" vertical="center"/>
+  </cellStyleXfs>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-  </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Bad" xfId="1" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="3" builtinId="23" customBuiltin="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Output" xfId="2" builtinId="21" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FF720E20"/>
-      <color rgb="FF162830"/>
+      <color rgb="FF711515"/>
+      <color rgb="FF9F1D1D"/>
     </mruColors>
   </colors>
   <extLst>
@@ -205,10 +164,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16C3C3E4-82F0-A046-B3C8-134BBFC8317D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -217,21 +176,15 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3766457" y="96018"/>
-          <a:ext cx="1458490" cy="581736"/>
+          <a:off x="3771259" y="96018"/>
+          <a:ext cx="1443442" cy="584937"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -539,16 +492,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE0AC16-40FD-4358-9BD0-D06EE6F324A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E71"/>
   <sheetFormatPr defaultColWidth="15.3046875" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="21.921875" customWidth="1"/>
-    <col min="2" max="2" width="36.23046875" customWidth="1"/>
-    <col min="3" max="3" width="36.53515625" customWidth="1"/>
-    <col min="4" max="4" width="20.84375" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="15.3046875" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="37" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="7" width="15.3046875" customWidth="1"/>
+    <col min="9" max="9" width="15.3046875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
@@ -559,44 +513,44 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="30" customHeight="1">
       <c r="A61" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="30" customHeight="1">
-      <c r="A71" s="1"/>
-      <c r="B71" s="1"/>
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="75" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" scale="75" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>